<commit_message>
update WCR dashboard data 2026-07-01 12:44
</commit_message>
<xml_diff>
--- a/docs/reports/daily/WCR_Kavach_Unified_KPI_Jun29-Jun29.xlsx
+++ b/docs/reports/daily/WCR_Kavach_Unified_KPI_Jun29-Jun29.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified KPI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Breakdown" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EB Detail" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Degradation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KM Verification" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Unified KPI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Daily Breakdown" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EB Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Mode Degradation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="KM Verification" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3270,7 +3270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L143"/>
+  <dimension ref="A1:M143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3348,6 +3348,11 @@
           <t>Valid Trip?</t>
         </is>
       </c>
+      <c r="M5" s="14" t="inlineStr">
+        <is>
+          <t>Loco Travel</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="31" t="inlineStr">
@@ -3404,6 +3409,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M6" s="16" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="31" t="inlineStr">
@@ -3460,6 +3466,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M7" s="16" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="31" t="inlineStr">
@@ -3516,6 +3523,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M8" s="16" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="31" t="inlineStr">
@@ -3572,6 +3580,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M9" s="16" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="31" t="inlineStr">
@@ -3628,6 +3637,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M10" s="16" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="31" t="inlineStr">
@@ -3684,6 +3694,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M11" s="16" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="31" t="inlineStr">
@@ -3740,6 +3751,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M12" s="16" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="31" t="inlineStr">
@@ -3796,6 +3808,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M13" s="16" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="31" t="inlineStr">
@@ -3852,6 +3865,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M14" s="16" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -3908,6 +3922,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M15" s="16" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="31" t="inlineStr">
@@ -3964,6 +3979,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M16" s="16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
@@ -4020,6 +4036,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M17" s="16" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -4076,6 +4093,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M18" s="16" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -4132,6 +4150,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M19" s="16" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="31" t="inlineStr">
@@ -4188,6 +4207,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M20" s="16" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
@@ -4244,6 +4264,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M21" s="16" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="31" t="inlineStr">
@@ -4300,6 +4321,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M22" s="16" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="31" t="inlineStr">
@@ -4356,6 +4378,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M23" s="16" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="31" t="inlineStr">
@@ -4412,6 +4435,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M24" s="16" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="31" t="inlineStr">
@@ -4468,6 +4492,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M25" s="16" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
@@ -4524,6 +4549,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M26" s="16" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="31" t="inlineStr">
@@ -4580,6 +4606,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M27" s="16" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="31" t="inlineStr">
@@ -4636,6 +4663,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M28" s="16" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="31" t="inlineStr">
@@ -4692,6 +4720,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M29" s="16" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="31" t="inlineStr">
@@ -4748,6 +4777,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M30" s="16" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
@@ -4804,6 +4834,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M31" s="16" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
@@ -4860,6 +4891,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M32" s="16" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -4916,6 +4948,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M33" s="16" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="31" t="inlineStr">
@@ -4972,6 +5005,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M34" s="16" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="31" t="inlineStr">
@@ -5028,6 +5062,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M35" s="16" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="31" t="inlineStr">
@@ -5084,6 +5119,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M36" s="16" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -5140,6 +5176,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M37" s="16" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -5196,6 +5233,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M38" s="16" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="31" t="inlineStr">
@@ -5252,6 +5290,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M39" s="16" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
@@ -5308,6 +5347,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M40" s="16" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="31" t="inlineStr">
@@ -5364,6 +5404,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M41" s="16" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
@@ -5420,6 +5461,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M42" s="16" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
@@ -5476,6 +5518,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M43" s="16" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="31" t="inlineStr">
@@ -5532,6 +5575,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M44" s="16" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
@@ -5588,6 +5632,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M45" s="16" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
@@ -5644,6 +5689,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M46" s="16" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
@@ -5700,6 +5746,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M47" s="16" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
@@ -5756,6 +5803,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M48" s="16" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
@@ -5812,6 +5860,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M49" s="16" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
@@ -5868,6 +5917,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M50" s="16" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
@@ -5924,6 +5974,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M51" s="16" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
@@ -5980,6 +6031,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M52" s="16" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="31" t="inlineStr">
@@ -6036,6 +6088,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M53" s="16" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
@@ -6092,6 +6145,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M54" s="16" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
@@ -6148,6 +6202,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M55" s="16" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
@@ -6204,6 +6259,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M56" s="16" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="31" t="inlineStr">
@@ -6260,6 +6316,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M57" s="16" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
@@ -6316,6 +6373,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M58" s="16" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
@@ -6372,6 +6430,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M59" s="16" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
@@ -6428,6 +6487,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M60" s="16" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="31" t="inlineStr">
@@ -6484,6 +6544,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M61" s="16" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="31" t="inlineStr">
@@ -6540,6 +6601,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M62" s="16" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="31" t="inlineStr">
@@ -6596,6 +6658,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M63" s="16" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="16" t="inlineStr">
@@ -6652,6 +6715,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M64" s="16" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
@@ -6708,6 +6772,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M65" s="16" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="31" t="inlineStr">
@@ -6764,6 +6829,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M66" s="16" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="16" t="inlineStr">
@@ -6820,6 +6886,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M67" s="16" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
@@ -6876,6 +6943,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M68" s="16" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
@@ -6932,6 +7000,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M69" s="16" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="16" t="inlineStr">
@@ -6988,6 +7057,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M70" s="16" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="16" t="inlineStr">
@@ -7044,6 +7114,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M71" s="16" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
@@ -7100,6 +7171,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M72" s="16" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="16" t="inlineStr">
@@ -7156,6 +7228,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M73" s="16" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr">
@@ -7212,6 +7285,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M74" s="16" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="16" t="inlineStr">
@@ -7268,6 +7342,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M75" s="16" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="16" t="inlineStr">
@@ -7324,6 +7399,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M76" s="16" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
@@ -7380,6 +7456,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M77" s="16" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="16" t="inlineStr">
@@ -7436,6 +7513,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M78" s="16" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="16" t="inlineStr">
@@ -7492,6 +7570,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M79" s="16" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
@@ -7548,6 +7627,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M80" s="16" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="16" t="inlineStr">
@@ -7604,6 +7684,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M81" s="16" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="16" t="inlineStr">
@@ -7660,6 +7741,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M82" s="16" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="16" t="inlineStr">
@@ -7716,6 +7798,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M83" s="16" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="16" t="inlineStr">
@@ -7772,6 +7855,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M84" s="16" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="16" t="inlineStr">
@@ -7828,6 +7912,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M85" s="16" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="16" t="inlineStr">
@@ -7884,6 +7969,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M86" s="16" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
@@ -7940,6 +8026,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M87" s="16" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="16" t="inlineStr">
@@ -7996,6 +8083,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M88" s="16" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="16" t="inlineStr">
@@ -8052,6 +8140,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M89" s="16" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="16" t="inlineStr">
@@ -8108,6 +8197,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M90" s="16" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="16" t="inlineStr">
@@ -8164,6 +8254,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M91" s="16" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="16" t="inlineStr">
@@ -8220,6 +8311,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M92" s="16" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="16" t="inlineStr">
@@ -8276,6 +8368,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M93" s="16" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="16" t="inlineStr">
@@ -8332,6 +8425,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M94" s="16" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="31" t="inlineStr">
@@ -8388,6 +8482,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M95" s="16" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="31" t="inlineStr">
@@ -8444,6 +8539,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M96" s="16" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="31" t="inlineStr">
@@ -8500,6 +8596,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M97" s="16" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
@@ -8556,6 +8653,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M98" s="16" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="16" t="inlineStr">
@@ -8612,6 +8710,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M99" s="16" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
@@ -8668,6 +8767,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M100" s="16" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
@@ -8724,6 +8824,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M101" s="16" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
@@ -8780,6 +8881,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M102" s="16" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
@@ -8836,6 +8938,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M103" s="16" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
@@ -8892,6 +8995,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M104" s="16" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="16" t="inlineStr">
@@ -8948,6 +9052,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M105" s="16" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
@@ -9004,6 +9109,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M106" s="16" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="16" t="inlineStr">
@@ -9060,6 +9166,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M107" s="16" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="16" t="inlineStr">
@@ -9116,6 +9223,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M108" s="16" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
@@ -9172,6 +9280,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M109" s="16" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="31" t="inlineStr">
@@ -9228,6 +9337,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M110" s="16" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="31" t="inlineStr">
@@ -9284,6 +9394,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M111" s="16" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="16" t="inlineStr">
@@ -9340,6 +9451,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M112" s="16" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="31" t="inlineStr">
@@ -9396,6 +9508,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M113" s="16" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="31" t="inlineStr">
@@ -9452,6 +9565,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M114" s="16" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="31" t="inlineStr">
@@ -9508,6 +9622,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M115" s="16" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="16" t="inlineStr">
@@ -9564,6 +9679,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M116" s="16" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="31" t="inlineStr">
@@ -9620,6 +9736,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M117" s="16" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="31" t="inlineStr">
@@ -9676,6 +9793,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M118" s="16" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="31" t="inlineStr">
@@ -9732,6 +9850,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M119" s="16" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="31" t="inlineStr">
@@ -9788,6 +9907,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M120" s="16" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="16" t="inlineStr">
@@ -9844,6 +9964,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M121" s="16" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="16" t="inlineStr">
@@ -9900,6 +10021,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M122" s="16" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="16" t="inlineStr">
@@ -9956,6 +10078,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M123" s="16" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="31" t="inlineStr">
@@ -10012,6 +10135,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M124" s="16" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="31" t="inlineStr">
@@ -10068,6 +10192,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M125" s="16" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="31" t="inlineStr">
@@ -10124,6 +10249,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M126" s="16" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="16" t="inlineStr">
@@ -10180,6 +10306,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M127" s="16" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="16" t="inlineStr">
@@ -10236,6 +10363,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M128" s="16" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="31" t="inlineStr">
@@ -10292,6 +10420,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M129" s="16" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="31" t="inlineStr">
@@ -10348,6 +10477,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M130" s="16" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="31" t="inlineStr">
@@ -10404,6 +10534,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M131" s="16" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="31" t="inlineStr">
@@ -10460,6 +10591,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M132" s="16" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="31" t="inlineStr">
@@ -10516,6 +10648,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M133" s="16" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="16" t="inlineStr">
@@ -10572,6 +10705,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M134" s="16" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="16" t="inlineStr">
@@ -10628,6 +10762,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M135" s="16" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="31" t="inlineStr">
@@ -10684,6 +10819,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M136" s="16" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="31" t="inlineStr">
@@ -10740,6 +10876,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M137" s="16" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="31" t="inlineStr">
@@ -10796,6 +10933,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M138" s="16" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="31" t="inlineStr">
@@ -10852,6 +10990,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M139" s="16" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="31" t="inlineStr">
@@ -10908,6 +11047,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M140" s="16" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="16" t="inlineStr">
@@ -10964,6 +11104,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M141" s="16" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="31" t="inlineStr">
@@ -11020,6 +11161,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M142" s="16" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="31" t="inlineStr">
@@ -11076,6 +11218,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M143" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
update WCR dashboard data 2026-07-01 13:00
</commit_message>
<xml_diff>
--- a/docs/reports/daily/WCR_Kavach_Unified_KPI_Jun29-Jun29.xlsx
+++ b/docs/reports/daily/WCR_Kavach_Unified_KPI_Jun29-Jun29.xlsx
@@ -3409,7 +3409,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M6" s="16" t="inlineStr"/>
+      <c r="M6" s="16" t="inlineStr">
+        <is>
+          <t>IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="31" t="inlineStr">
@@ -3466,7 +3470,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M7" s="16" t="inlineStr"/>
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="31" t="inlineStr">
@@ -3523,7 +3531,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M8" s="16" t="inlineStr"/>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="31" t="inlineStr">
@@ -3580,7 +3592,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M9" s="16" t="inlineStr"/>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="31" t="inlineStr">
@@ -3637,7 +3653,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M10" s="16" t="inlineStr"/>
+      <c r="M10" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="31" t="inlineStr">
@@ -3694,7 +3714,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M11" s="16" t="inlineStr"/>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="31" t="inlineStr">
@@ -3751,7 +3775,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M12" s="16" t="inlineStr"/>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="31" t="inlineStr">
@@ -3808,7 +3836,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M13" s="16" t="inlineStr"/>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="31" t="inlineStr">
@@ -3865,7 +3897,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M14" s="16" t="inlineStr"/>
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -3922,7 +3958,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M15" s="16" t="inlineStr"/>
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="31" t="inlineStr">
@@ -3979,7 +4019,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M16" s="16" t="inlineStr"/>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
@@ -4036,7 +4080,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M17" s="16" t="inlineStr"/>
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -4093,7 +4141,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M18" s="16" t="inlineStr"/>
+      <c r="M18" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -4150,7 +4202,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M19" s="16" t="inlineStr"/>
+      <c r="M19" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="31" t="inlineStr">
@@ -4207,7 +4263,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M20" s="16" t="inlineStr"/>
+      <c r="M20" s="16" t="inlineStr">
+        <is>
+          <t>NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="31" t="inlineStr">
@@ -4264,7 +4324,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M21" s="16" t="inlineStr"/>
+      <c r="M21" s="16" t="inlineStr">
+        <is>
+          <t>NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="31" t="inlineStr">
@@ -4321,7 +4385,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M22" s="16" t="inlineStr"/>
+      <c r="M22" s="16" t="inlineStr">
+        <is>
+          <t>NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="31" t="inlineStr">
@@ -4378,7 +4446,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M23" s="16" t="inlineStr"/>
+      <c r="M23" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="31" t="inlineStr">
@@ -4435,7 +4507,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M24" s="16" t="inlineStr"/>
+      <c r="M24" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="31" t="inlineStr">
@@ -4492,7 +4568,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M25" s="16" t="inlineStr"/>
+      <c r="M25" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
@@ -4549,7 +4629,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M26" s="16" t="inlineStr"/>
+      <c r="M26" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="31" t="inlineStr">
@@ -4606,7 +4690,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M27" s="16" t="inlineStr"/>
+      <c r="M27" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="31" t="inlineStr">
@@ -4663,7 +4751,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M28" s="16" t="inlineStr"/>
+      <c r="M28" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="31" t="inlineStr">
@@ -4720,7 +4812,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M29" s="16" t="inlineStr"/>
+      <c r="M29" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="31" t="inlineStr">
@@ -4777,7 +4873,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M30" s="16" t="inlineStr"/>
+      <c r="M30" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
@@ -4834,7 +4934,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M31" s="16" t="inlineStr"/>
+      <c r="M31" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
@@ -4891,7 +4995,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M32" s="16" t="inlineStr"/>
+      <c r="M32" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -4948,7 +5056,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M33" s="16" t="inlineStr"/>
+      <c r="M33" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="31" t="inlineStr">
@@ -5005,7 +5117,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M34" s="16" t="inlineStr"/>
+      <c r="M34" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="31" t="inlineStr">
@@ -5062,7 +5178,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M35" s="16" t="inlineStr"/>
+      <c r="M35" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="31" t="inlineStr">
@@ -5119,7 +5239,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M36" s="16" t="inlineStr"/>
+      <c r="M36" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -5176,7 +5300,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M37" s="16" t="inlineStr"/>
+      <c r="M37" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -5233,7 +5361,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M38" s="16" t="inlineStr"/>
+      <c r="M38" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="31" t="inlineStr">
@@ -5290,7 +5422,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M39" s="16" t="inlineStr"/>
+      <c r="M39" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
@@ -5347,7 +5483,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M40" s="16" t="inlineStr"/>
+      <c r="M40" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="31" t="inlineStr">
@@ -5404,7 +5544,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M41" s="16" t="inlineStr"/>
+      <c r="M41" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="16" t="inlineStr">
@@ -5461,7 +5605,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M42" s="16" t="inlineStr"/>
+      <c r="M42" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
@@ -5518,7 +5666,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M43" s="16" t="inlineStr"/>
+      <c r="M43" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="31" t="inlineStr">
@@ -5575,7 +5727,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M44" s="16" t="inlineStr"/>
+      <c r="M44" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
@@ -5632,7 +5788,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M45" s="16" t="inlineStr"/>
+      <c r="M45" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
@@ -5689,7 +5849,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M46" s="16" t="inlineStr"/>
+      <c r="M46" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
@@ -5746,7 +5910,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M47" s="16" t="inlineStr"/>
+      <c r="M47" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
@@ -5803,7 +5971,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M48" s="16" t="inlineStr"/>
+      <c r="M48" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
@@ -5860,7 +6032,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M49" s="16" t="inlineStr"/>
+      <c r="M49" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
@@ -5917,7 +6093,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M50" s="16" t="inlineStr"/>
+      <c r="M50" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
@@ -5974,7 +6154,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M51" s="16" t="inlineStr"/>
+      <c r="M51" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
@@ -6031,7 +6215,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M52" s="16" t="inlineStr"/>
+      <c r="M52" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="31" t="inlineStr">
@@ -6088,7 +6276,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M53" s="16" t="inlineStr"/>
+      <c r="M53" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="31" t="inlineStr">
@@ -6145,7 +6337,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M54" s="16" t="inlineStr"/>
+      <c r="M54" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
@@ -6202,7 +6398,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M55" s="16" t="inlineStr"/>
+      <c r="M55" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
@@ -6259,7 +6459,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M56" s="16" t="inlineStr"/>
+      <c r="M56" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="31" t="inlineStr">
@@ -6316,7 +6520,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M57" s="16" t="inlineStr"/>
+      <c r="M57" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
@@ -6373,7 +6581,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M58" s="16" t="inlineStr"/>
+      <c r="M58" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
@@ -6430,7 +6642,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M59" s="16" t="inlineStr"/>
+      <c r="M59" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
@@ -6487,7 +6703,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M60" s="16" t="inlineStr"/>
+      <c r="M60" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="31" t="inlineStr">
@@ -6544,7 +6764,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M61" s="16" t="inlineStr"/>
+      <c r="M61" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="31" t="inlineStr">
@@ -6601,7 +6825,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M62" s="16" t="inlineStr"/>
+      <c r="M62" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="31" t="inlineStr">
@@ -6658,7 +6886,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M63" s="16" t="inlineStr"/>
+      <c r="M63" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="16" t="inlineStr">
@@ -6715,7 +6947,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M64" s="16" t="inlineStr"/>
+      <c r="M64" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
@@ -6772,7 +7008,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M65" s="16" t="inlineStr"/>
+      <c r="M65" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="31" t="inlineStr">
@@ -6829,7 +7069,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M66" s="16" t="inlineStr"/>
+      <c r="M66" s="16" t="inlineStr">
+        <is>
+          <t>IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="16" t="inlineStr">
@@ -6886,7 +7130,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M67" s="16" t="inlineStr"/>
+      <c r="M67" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
@@ -6943,7 +7191,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M68" s="16" t="inlineStr"/>
+      <c r="M68" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
@@ -7000,7 +7252,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M69" s="16" t="inlineStr"/>
+      <c r="M69" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="16" t="inlineStr">
@@ -7057,7 +7313,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M70" s="16" t="inlineStr"/>
+      <c r="M70" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="16" t="inlineStr">
@@ -7114,7 +7374,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M71" s="16" t="inlineStr"/>
+      <c r="M71" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
@@ -7171,7 +7435,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M72" s="16" t="inlineStr"/>
+      <c r="M72" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="16" t="inlineStr">
@@ -7228,7 +7496,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M73" s="16" t="inlineStr"/>
+      <c r="M73" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr">
@@ -7285,7 +7557,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M74" s="16" t="inlineStr"/>
+      <c r="M74" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="16" t="inlineStr">
@@ -7342,7 +7618,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M75" s="16" t="inlineStr"/>
+      <c r="M75" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="16" t="inlineStr">
@@ -7399,7 +7679,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M76" s="16" t="inlineStr"/>
+      <c r="M76" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
@@ -7456,7 +7740,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M77" s="16" t="inlineStr"/>
+      <c r="M77" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="16" t="inlineStr">
@@ -7513,7 +7801,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M78" s="16" t="inlineStr"/>
+      <c r="M78" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="16" t="inlineStr">
@@ -7570,7 +7862,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M79" s="16" t="inlineStr"/>
+      <c r="M79" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
@@ -7627,7 +7923,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M80" s="16" t="inlineStr"/>
+      <c r="M80" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="16" t="inlineStr">
@@ -7684,7 +7984,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M81" s="16" t="inlineStr"/>
+      <c r="M81" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="16" t="inlineStr">
@@ -7741,7 +8045,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M82" s="16" t="inlineStr"/>
+      <c r="M82" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="16" t="inlineStr">
@@ -7798,7 +8106,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M83" s="16" t="inlineStr"/>
+      <c r="M83" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="16" t="inlineStr">
@@ -7855,7 +8167,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M84" s="16" t="inlineStr"/>
+      <c r="M84" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="16" t="inlineStr">
@@ -7912,7 +8228,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M85" s="16" t="inlineStr"/>
+      <c r="M85" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="16" t="inlineStr">
@@ -7969,7 +8289,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M86" s="16" t="inlineStr"/>
+      <c r="M86" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
@@ -8026,7 +8350,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M87" s="16" t="inlineStr"/>
+      <c r="M87" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="16" t="inlineStr">
@@ -8083,7 +8411,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M88" s="16" t="inlineStr"/>
+      <c r="M88" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="16" t="inlineStr">
@@ -8140,7 +8472,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M89" s="16" t="inlineStr"/>
+      <c r="M89" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="16" t="inlineStr">
@@ -8197,7 +8533,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M90" s="16" t="inlineStr"/>
+      <c r="M90" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="16" t="inlineStr">
@@ -8254,7 +8594,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M91" s="16" t="inlineStr"/>
+      <c r="M91" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="16" t="inlineStr">
@@ -8311,7 +8655,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M92" s="16" t="inlineStr"/>
+      <c r="M92" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="16" t="inlineStr">
@@ -8368,7 +8716,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M93" s="16" t="inlineStr"/>
+      <c r="M93" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="16" t="inlineStr">
@@ -8425,7 +8777,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M94" s="16" t="inlineStr"/>
+      <c r="M94" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="31" t="inlineStr">
@@ -8482,7 +8838,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M95" s="16" t="inlineStr"/>
+      <c r="M95" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="31" t="inlineStr">
@@ -8539,7 +8899,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M96" s="16" t="inlineStr"/>
+      <c r="M96" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="31" t="inlineStr">
@@ -8596,7 +8960,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M97" s="16" t="inlineStr"/>
+      <c r="M97" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
@@ -8653,7 +9021,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M98" s="16" t="inlineStr"/>
+      <c r="M98" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="16" t="inlineStr">
@@ -8710,7 +9082,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M99" s="16" t="inlineStr"/>
+      <c r="M99" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
@@ -8767,7 +9143,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M100" s="16" t="inlineStr"/>
+      <c r="M100" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="31" t="inlineStr">
@@ -8824,7 +9204,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M101" s="16" t="inlineStr"/>
+      <c r="M101" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="inlineStr">
@@ -8881,7 +9265,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M102" s="16" t="inlineStr"/>
+      <c r="M102" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="31" t="inlineStr">
@@ -8938,7 +9326,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M103" s="16" t="inlineStr"/>
+      <c r="M103" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="31" t="inlineStr">
@@ -8995,7 +9387,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M104" s="16" t="inlineStr"/>
+      <c r="M104" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="16" t="inlineStr">
@@ -9052,7 +9448,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M105" s="16" t="inlineStr"/>
+      <c r="M105" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
@@ -9109,7 +9509,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M106" s="16" t="inlineStr"/>
+      <c r="M106" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="16" t="inlineStr">
@@ -9166,7 +9570,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M107" s="16" t="inlineStr"/>
+      <c r="M107" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="16" t="inlineStr">
@@ -9223,7 +9631,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M108" s="16" t="inlineStr"/>
+      <c r="M108" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
@@ -9280,7 +9692,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M109" s="16" t="inlineStr"/>
+      <c r="M109" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="31" t="inlineStr">
@@ -9337,7 +9753,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M110" s="16" t="inlineStr"/>
+      <c r="M110" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="31" t="inlineStr">
@@ -9394,7 +9814,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M111" s="16" t="inlineStr"/>
+      <c r="M111" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="16" t="inlineStr">
@@ -9451,7 +9875,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M112" s="16" t="inlineStr"/>
+      <c r="M112" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="31" t="inlineStr">
@@ -9508,7 +9936,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M113" s="16" t="inlineStr"/>
+      <c r="M113" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="31" t="inlineStr">
@@ -9565,7 +9997,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M114" s="16" t="inlineStr"/>
+      <c r="M114" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="31" t="inlineStr">
@@ -9622,7 +10058,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M115" s="16" t="inlineStr"/>
+      <c r="M115" s="16" t="inlineStr">
+        <is>
+          <t>SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="16" t="inlineStr">
@@ -9679,7 +10119,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M116" s="16" t="inlineStr"/>
+      <c r="M116" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="31" t="inlineStr">
@@ -9736,7 +10180,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M117" s="16" t="inlineStr"/>
+      <c r="M117" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="31" t="inlineStr">
@@ -9793,7 +10241,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M118" s="16" t="inlineStr"/>
+      <c r="M118" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="31" t="inlineStr">
@@ -9850,7 +10302,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M119" s="16" t="inlineStr"/>
+      <c r="M119" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="31" t="inlineStr">
@@ -9907,7 +10363,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M120" s="16" t="inlineStr"/>
+      <c r="M120" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="16" t="inlineStr">
@@ -9964,7 +10424,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M121" s="16" t="inlineStr"/>
+      <c r="M121" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="16" t="inlineStr">
@@ -10021,7 +10485,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M122" s="16" t="inlineStr"/>
+      <c r="M122" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="16" t="inlineStr">
@@ -10078,7 +10546,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M123" s="16" t="inlineStr"/>
+      <c r="M123" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="31" t="inlineStr">
@@ -10135,7 +10607,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M124" s="16" t="inlineStr"/>
+      <c r="M124" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="31" t="inlineStr">
@@ -10192,7 +10668,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M125" s="16" t="inlineStr"/>
+      <c r="M125" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="31" t="inlineStr">
@@ -10249,7 +10729,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M126" s="16" t="inlineStr"/>
+      <c r="M126" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="16" t="inlineStr">
@@ -10306,7 +10790,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M127" s="16" t="inlineStr"/>
+      <c r="M127" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="16" t="inlineStr">
@@ -10363,7 +10851,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M128" s="16" t="inlineStr"/>
+      <c r="M128" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="31" t="inlineStr">
@@ -10420,7 +10912,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M129" s="16" t="inlineStr"/>
+      <c r="M129" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="31" t="inlineStr">
@@ -10477,7 +10973,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M130" s="16" t="inlineStr"/>
+      <c r="M130" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="31" t="inlineStr">
@@ -10534,7 +11034,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M131" s="16" t="inlineStr"/>
+      <c r="M131" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="31" t="inlineStr">
@@ -10591,7 +11095,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M132" s="16" t="inlineStr"/>
+      <c r="M132" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="31" t="inlineStr">
@@ -10648,7 +11156,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M133" s="16" t="inlineStr"/>
+      <c r="M133" s="16" t="inlineStr">
+        <is>
+          <t>RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="16" t="inlineStr">
@@ -10705,7 +11217,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M134" s="16" t="inlineStr"/>
+      <c r="M134" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="16" t="inlineStr">
@@ -10762,7 +11278,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M135" s="16" t="inlineStr"/>
+      <c r="M135" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="31" t="inlineStr">
@@ -10819,7 +11339,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M136" s="16" t="inlineStr"/>
+      <c r="M136" s="16" t="inlineStr">
+        <is>
+          <t>VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="31" t="inlineStr">
@@ -10876,7 +11400,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M137" s="16" t="inlineStr"/>
+      <c r="M137" s="16" t="inlineStr">
+        <is>
+          <t>Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="31" t="inlineStr">
@@ -10933,7 +11461,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M138" s="16" t="inlineStr"/>
+      <c r="M138" s="16" t="inlineStr">
+        <is>
+          <t>Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="31" t="inlineStr">
@@ -10990,7 +11522,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M139" s="16" t="inlineStr"/>
+      <c r="M139" s="16" t="inlineStr">
+        <is>
+          <t>Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="31" t="inlineStr">
@@ -11047,7 +11583,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M140" s="16" t="inlineStr"/>
+      <c r="M140" s="16" t="inlineStr">
+        <is>
+          <t>Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="16" t="inlineStr">
@@ -11104,7 +11644,11 @@
           <t>Valid</t>
         </is>
       </c>
-      <c r="M141" s="16" t="inlineStr"/>
+      <c r="M141" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265, Murhesi Rampur(MSRP), IBH/LC-258, Jajjanpatti(JJA), DhaurmuiJaghina(DUM), IBH-247, Bharatpur Jn.(BTE), IBH-242, Sewar(SWAR), IBH-JCU, LC-232, Pingora(PNGR), IBH-229, 2.35 KM from KEV, Kela Devi(KEV), IBH-224, Bayana Jn.(BXN), LC-219, LC-217, IBH-216, Dumariya(DY), IBH-211, FatehSinghpura(FSP), IBH-DNHK, Hindaun City(HAN), LC-199, IBS-198, Shri Mahabirji(SMBJ), IBH-192, Piloda(PDZ), ChhotiOdai(COO), 8.375 KM from GGC, IBH-180, Gangapur City(GGC), Lalpur Umri(LRU), IBH/LC-173, NarayanpurTatwara(NNW), IBH-171, Nimoda(NMD), 3.5 KM from MLZ, Malarna(MLZ), IBH-MXL, LC-163, Makholi(MXL), IBH-159, Ranthambhor(RNT), 5.0 KM from SWM-A, SawaiMadhopurJn(SWM), LC-148, Kushtala(KTA), IBH-RWJ, 2.0 KM from RWJ, RawanjnaDungar(RWJ), 6.25 KM from AMLI, Amli(AMLI), IBH-140, IndragarhSumerganjMandi(IDG), LC-137, IBH-LKE, Lakheri(LKE), LC-136W, Laban(LBN), IBH-LBN, Ghatkavarana(GKB), IBH-131, LC-128, Kapren(KPZ), LC-126, IBH-125, Arnetha(ARE), LC-120, IBH-119, LC-118, KeshoraiPatan(KPTN), 2.75 KM from GQL (LC-113), Gurla(GQL), KOTA C, Kota Jn.(KOTA) CENTRAL, KOTA SOUTH, DakaniyaTalav(DKNT), Dadhdevi(DDV), ALNI/DDV, Alniya(ALNI), IBH DHANIKASAR, Ravtha Road(RDT), IBH-95(7.25KM FROM DARA), Dara(DARA), IBH KIW-DARA, Kanwalpura(KIW), 2.85 KM from MKX, Morak(MKX), IBH RMA-MKX, RamganjMandi(RMA), IBH-79, Jhalawar Road(JHW), DhuanKheri(DKRA), IBH-69, Bhawani Mandi(BWM), IBH-61(LC-60), Kurlasi(KRLS), IBH-55(7.5KM from GOH), Garoth(GOH), IBH-48, Shamgarh(SGZ), 3.0 Km From SGZ, IBH-HNU, Suwasra(SVA), NathuKheri(NKH), 4.5 KM from CMU, Chau Mahla(CMU), Talavli(TLZ), LC-28, IBH-27, Thuria(THUR), IBH-23, VikramgarhA lot(VMA), IBH-17, LuniRichha(LNR), IBH-10, Mehidpur Road(MEP), 3.9 KM  from RLK, Rohalkhurd(RLK), LC-3, IBH-1</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="31" t="inlineStr">
@@ -11161,7 +11705,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M142" s="16" t="inlineStr"/>
+      <c r="M142" s="16" t="inlineStr">
+        <is>
+          <t>KOTA C, Kota Jn.(KOTA) CENTRAL</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="31" t="inlineStr">
@@ -11218,7 +11766,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
-      <c r="M143" s="16" t="inlineStr"/>
+      <c r="M143" s="16" t="inlineStr">
+        <is>
+          <t>IBH 265</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>